<commit_message>
fix(frontend): R5 I1 재제출 조건 보완
</commit_message>
<xml_diff>
--- a/docs/deliverables/01_요구사항정의서_29기_3팀.xlsx
+++ b/docs/deliverables/01_요구사항정의서_29기_3팀.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시트1" sheetId="1" r:id="Rfc4eef8ee5ff4c8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시트1" sheetId="1" r:id="R0f79ae1ef5684242"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1147,7 +1147,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="160" t="str">
-        <x:v>DataHub Core 기반 대화형 데이터 분석·자동 리포팅 서비스 | SK네트웍스 Family AI 캠프 29기 3팀 | v1.2 | 기준일 2026-07-30 | 추적 요구사항 75개</x:v>
+        <x:v>DataHub Core 기반 대화형 데이터 분석·자동 리포팅 서비스 | SK네트웍스 Family AI 캠프 29기 3팀 | v1.1 | 기준일 2026-07-30 | 추적 요구사항 75개</x:v>
       </x:c>
       <x:c r="B2" s="160"/>
       <x:c r="C2" s="160"/>
@@ -4285,13 +4285,13 @@
         <x:v>REQ-SCP-001</x:v>
       </x:c>
       <x:c r="E77" s="208" t="str">
-        <x:v>MCP·문서 RAG·ML-as-a-Tool은 I5 이후 R1의 별도 일정·계약·비용·보안 Gate 승인 전 비활성 상태여야 한다.</x:v>
+        <x:v>MCP·문서 RAG·ML-as-a-Tool은 P0/P1 완료와 R1 편입 승인 전 비활성 상태여야 한다.</x:v>
       </x:c>
       <x:c r="F77" s="208" t="str">
-        <x:v>route·메뉴·worker·dependency를 선행 구현하지 않고 현재 P0/P1·I5 완료율을 차단하지 않는다.</x:v>
+        <x:v>route·메뉴·worker·dependency를 선행 구현하지 않는다.</x:v>
       </x:c>
       <x:c r="G77" s="208" t="str">
-        <x:v>P2·후속 대기</x:v>
+        <x:v>P2·기본 제외</x:v>
       </x:c>
       <x:c r="H77"/>
       <x:c r="I77"/>
@@ -4327,13 +4327,13 @@
         <x:v>REQ-SCP-002</x:v>
       </x:c>
       <x:c r="E78" s="208" t="str">
-        <x:v>고객 360은 I5 이후 identity mapping·masking·전용 권한·감사·별도 수용 기준 승인 전 비활성 상태여야 한다.</x:v>
+        <x:v>고객 360은 identity mapping·masking·전용 권한과 일정 영향 승인 전 비활성 상태여야 한다.</x:v>
       </x:c>
       <x:c r="F78" s="208" t="str">
-        <x:v>승인 전 MVP navigation과 직접 route에서 접근할 수 없고 현재 P0/P1·I5 완료율을 차단하지 않는다.</x:v>
+        <x:v>승인 전 MVP navigation과 직접 route에서 접근할 수 없다.</x:v>
       </x:c>
       <x:c r="G78" s="208" t="str">
-        <x:v>후속 대기</x:v>
+        <x:v>선택·기본 제외</x:v>
       </x:c>
       <x:c r="H78"/>
       <x:c r="I78"/>
@@ -4369,13 +4369,13 @@
         <x:v>REQ-SCP-003</x:v>
       </x:c>
       <x:c r="E79" s="208" t="str">
-        <x:v>외부 Report 배포와 다단 승인 workflow는 I5 이후 별도 Gate 승인 전 구현하지 않아야 한다.</x:v>
+        <x:v>외부 Report 배포와 다단 승인 workflow는 별도 승인 전 구현하지 않아야 한다.</x:v>
       </x:c>
       <x:c r="F79" s="208" t="str">
         <x:v>P0는 내부 정의·승인·수동/스케줄 실행·이력에 한정한다.</x:v>
       </x:c>
       <x:c r="G79" s="208" t="str">
-        <x:v>P2·후속 대기</x:v>
+        <x:v>P2·기본 제외</x:v>
       </x:c>
       <x:c r="H79"/>
       <x:c r="I79"/>

</xml_diff>